<commit_message>
Add new Excel file for modified undergraduate data
</commit_message>
<xml_diff>
--- a/data/novedades/Modificados_posgrado.xlsx
+++ b/data/novedades/Modificados_posgrado.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN1"/>
+  <dimension ref="A1:Y9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,107 +530,920 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>CÓDIGO_INSTITUCIÓN_ANTERIOR</t>
+          <t>PROGINSTI</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>NOMBRE_INSTITUCIÓN_ANTERIOR</t>
+          <t>NÚMERO_CRÉDITOS_NUEVOS</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>SECTOR_ANTERIOR</t>
+          <t>NÚMERO_CRÉDITOS_ANTERIORES</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>DEPARTAMENTO_OFERTA_PROGRAMA_ANTERIOR</t>
+          <t>FECHA_OBTENCION</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>MUNICIPIO_OFERTA_PROGRAMA_ANTERIOR</t>
+          <t>DIVISIÓN UNINORTE</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>NOMBRE_DEL_PROGRAMA_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>MODALIDAD_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>NÚMERO_CRÉDITOS_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>NÚMERO_PERIODOS_DE_DURACIÓN_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>PERIODICIDAD_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>COSTO_MATRÍCULA_ESTUD_NUEVOS_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>PERIODICIDAD_ADMISIONES_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>FECHA_DE_REGISTRO_EN_SNIES_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>CINE_F_2013_AC_CAMPO_AMPLIO_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>CINE_F_2013_AC_CAMPO_ESPECÍFIC_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>CINE_F_2013_AC_CAMPO_DETALLADO_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>NÚCLEO_BÁSICO_DEL_CONOCIMIENTO_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>NIVEL_DE_FORMACIÓN_ANTERIOR</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>FECHA_DETECCION</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>DIVISIÓN UNINORTE</t>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6569</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN CARDIOLOGIA PEDIATRICA</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>121</v>
+      </c>
+      <c r="J2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>31697659</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Por cohorte</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>44572</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>6569-121</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>130</v>
+      </c>
+      <c r="V2" t="n">
+        <v>121</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>104918</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACIÓN EN CIRUGIA DE MANO</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>54</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>29503364</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>44755</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>104918-54</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
+        <v>64</v>
+      </c>
+      <c r="V3" t="n">
+        <v>54</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1319</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN ENDOCRINOLOGIA</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>114</v>
+      </c>
+      <c r="J4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>31697659</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>44299</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>1319-114</t>
+        </is>
+      </c>
+      <c r="U4" t="n">
+        <v>97</v>
+      </c>
+      <c r="V4" t="n">
+        <v>114</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1305</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN GINECOLOGIA Y OBSTETRICIA</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>208</v>
+      </c>
+      <c r="J5" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>31697659</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>44295</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>1305-208</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>270</v>
+      </c>
+      <c r="V5" t="n">
+        <v>208</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>104922</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACIÓN EN MASTOLOGÍA</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>117</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>29503364</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>44725</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>104922-117</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>104</v>
+      </c>
+      <c r="V6" t="n">
+        <v>117</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>16130</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN MEDICINA MATERNO FETAL</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>125</v>
+      </c>
+      <c r="J7" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>27306068</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>44671</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>16130-125</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>130</v>
+      </c>
+      <c r="V7" t="n">
+        <v>125</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1308</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN NEFROLOGIA</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>119</v>
+      </c>
+      <c r="J8" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>31697659</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>44299</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>1308-119</t>
+        </is>
+      </c>
+      <c r="U8" t="n">
+        <v>88</v>
+      </c>
+      <c r="V8" t="n">
+        <v>119</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1714</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>COLEGIO MAYOR DE NUESTRA SEÑORA DEL ROSARIO</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>1315</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ESPECIALIZACION EN PEDIATRIA</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>282</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>31697659</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>44292</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Especialización médico quirúrgica</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>1315-282</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>182</v>
+      </c>
+      <c r="V9" t="n">
+        <v>282</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>02/07/2025</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Activo</t>
         </is>
       </c>
     </row>

</xml_diff>